<commit_message>
Complete image category normalization across all tracked files
Fix remaining non-canonical image_category values missed in previous
commit. The prior fix only covered per-year JSON + some XLSX files.

This commit normalizes all remaining occurrences:
- Dataset/EN/ITAMed_Distribution_EN.xlsx (3 sheets, 24->21 categories)
- Dataset/IT/ITAMed_Distribution_IT.xlsx (3 sheets, 24->21 categories)
- Dataset/EN/xlsx/ITAMed_2023_EN.xlsx ('Endoscopic image ' trailing ws)
- Dataset/EN/xlsx/ITAMed_complete_EN.xlsx (same)
- Dataset/IT/xlsx/ITAMed_2023.xlsx (same)
- Dataset_Translation/ITAMed_complete_EN_tracked.xlsx (3 aliases)

Aliases resolved:
- 'Endoscopic image ' -> 'Endoscopic image' (trailing whitespace)
- 'Brain CT Scan' -> 'Brain CT scan' (case normalization)
- 'Brain TC scan' -> 'Brain CT scan' (Italian TC = English CT)

Verified: 0 problems across all JSON + XLSX files in the entire repo.
Pipeline validation passes all 13 checks including image vocabulary.
</commit_message>
<xml_diff>
--- a/Dataset/EN/ITAMed_Distribution_EN.xlsx
+++ b/Dataset/EN/ITAMed_Distribution_EN.xlsx
@@ -2989,7 +2989,7 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Brain CT Scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Endoscopic image </t>
+          <t>Endoscopic image</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Brain TC scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
@@ -4478,7 +4478,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Brain CT Scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -4589,7 +4589,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Endoscopic image </t>
+          <t>Endoscopic image</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -4663,7 +4663,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Brain TC scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Brain CT Scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -5513,7 +5513,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Endoscopic image </t>
+          <t>Endoscopic image</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -5539,7 +5539,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Brain TC scan</t>
+          <t>Brain CT scan</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">

</xml_diff>